<commit_message>
added dataanalysis for hydrogen use in sectors
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-ships.xlsx
+++ b/premise/data/additional_inventories/lci-ships.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA23D2A4-BEA8-4936-BBFE-826CDCD39D6A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46B79077-8F25-4DC2-B2E2-0B7C8F7DAEBC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10500" yWindow="660" windowWidth="25824" windowHeight="18984" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2490,8 +2490,8 @@
         <v>4.5451388888888888E-8</v>
       </c>
       <c r="K84" s="6">
-        <f t="shared" ref="K84:K86" si="2">0.00002*(B77*18.6*B72/3.6)</f>
-        <v>1.6145833333333334E-12</v>
+        <f>0.00002*(B76*18.6*B71/3.6)</f>
+        <v>2.5812601273148154E-7</v>
       </c>
       <c r="L84" s="6">
         <f>0.0000028*(B76*18.6*B72/3.6)</f>
@@ -2526,8 +2526,8 @@
         <v>6.4930555555555568E-7</v>
       </c>
       <c r="K85" s="6">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>0.00002*(B76*18.6*B71/3.6)</f>
+        <v>2.5812601273148154E-7</v>
       </c>
       <c r="L85" s="6">
         <f>0.00004*(B76*18.6*B72/3.6)</f>
@@ -2561,9 +2561,9 @@
         <f t="shared" si="1"/>
         <v>7.4670138888888891E-7</v>
       </c>
-      <c r="K86" s="6" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
+      <c r="K86" s="6">
+        <f>0.00002*(B76*18.6*B71/3.6)</f>
+        <v>2.5812601273148154E-7</v>
       </c>
       <c r="L86">
         <f>0.00013*(B76*18.6*B72/3.6)</f>
@@ -2979,7 +2979,7 @@
         <v>5</v>
       </c>
       <c r="J112" s="6">
-        <f t="shared" ref="J112:J115" si="3">B112</f>
+        <f t="shared" ref="J112:J115" si="2">B112</f>
         <v>7.7916666666666672E-5</v>
       </c>
       <c r="K112" s="6">
@@ -3015,7 +3015,7 @@
         <v>5</v>
       </c>
       <c r="J113" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>9.3613953124999986E-5</v>
       </c>
       <c r="K113" s="6">
@@ -3051,7 +3051,7 @@
         <v>5</v>
       </c>
       <c r="J114" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>4.2035554687499993E-5</v>
       </c>
       <c r="K114" s="6">
@@ -3087,7 +3087,7 @@
         <v>5</v>
       </c>
       <c r="J115" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>7.953993055555555E-9</v>
       </c>
       <c r="K115" s="6">
@@ -3509,7 +3509,7 @@
         <v>5</v>
       </c>
       <c r="J141" s="6">
-        <f t="shared" ref="J141:J144" si="4">B141</f>
+        <f t="shared" ref="J141:J144" si="3">B141</f>
         <v>4.0680701754385975E-5</v>
       </c>
       <c r="K141" s="6">
@@ -3545,7 +3545,7 @@
         <v>5</v>
       </c>
       <c r="J142" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.5589473684210534E-5</v>
       </c>
       <c r="K142" s="6">
@@ -3581,7 +3581,7 @@
         <v>5</v>
       </c>
       <c r="J143" s="6">
-        <f t="shared" ref="J143" si="5">B143</f>
+        <f t="shared" ref="J143" si="4">B143</f>
         <v>6.5614035087719314E-7</v>
       </c>
       <c r="K143" s="6">
@@ -3617,7 +3617,7 @@
         <v>5</v>
       </c>
       <c r="J144" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>6.5614035087719314E-7</v>
       </c>
       <c r="K144" s="6">
@@ -3653,7 +3653,7 @@
         <v>5</v>
       </c>
       <c r="J145" s="6">
-        <f t="shared" ref="J145:J147" si="6">B145</f>
+        <f t="shared" ref="J145:J147" si="5">B145</f>
         <v>6.6488888888888891E-5</v>
       </c>
       <c r="K145" s="6">
@@ -3689,7 +3689,7 @@
         <v>5</v>
       </c>
       <c r="J146" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>8.311111111111113E-6</v>
       </c>
       <c r="K146" s="6">
@@ -3725,7 +3725,7 @@
         <v>5</v>
       </c>
       <c r="J147" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>4.3742690058479546E-7</v>
       </c>
       <c r="K147" s="11">
@@ -4142,7 +4142,7 @@
         <v>5</v>
       </c>
       <c r="J174" s="6">
-        <f t="shared" ref="J174:J180" si="7">B174</f>
+        <f t="shared" ref="J174:J180" si="6">B174</f>
         <v>2.6523108669611446E-5</v>
       </c>
       <c r="K174" s="6">
@@ -4178,7 +4178,7 @@
         <v>5</v>
       </c>
       <c r="J175" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1.6683890937336232E-5</v>
       </c>
       <c r="K175" s="6">
@@ -4214,7 +4214,7 @@
         <v>5</v>
       </c>
       <c r="J176" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>4.2779207531631361E-7</v>
       </c>
       <c r="K176" s="6">
@@ -4250,7 +4250,7 @@
         <v>5</v>
       </c>
       <c r="J177" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>4.2779207531631361E-7</v>
       </c>
       <c r="K177" s="6">
@@ -4286,7 +4286,7 @@
         <v>5</v>
       </c>
       <c r="J178" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>4.5234362050838021E-5</v>
       </c>
       <c r="K178" s="6">
@@ -4322,7 +4322,7 @@
         <v>5</v>
       </c>
       <c r="J179" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>5.4186996206733058E-6</v>
       </c>
       <c r="K179" s="6">
@@ -4358,7 +4358,7 @@
         <v>5</v>
       </c>
       <c r="J180" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>2.8519471687754242E-7</v>
       </c>
       <c r="K180" s="11">
@@ -4748,7 +4748,7 @@
         <v>5</v>
       </c>
       <c r="J206" s="6">
-        <f t="shared" ref="J206" si="8">B206</f>
+        <f t="shared" ref="J206" si="7">B206</f>
         <v>1.0925271739130437E-5</v>
       </c>
       <c r="K206" s="6">
@@ -4784,7 +4784,7 @@
         <v>5</v>
       </c>
       <c r="J207" s="6">
-        <f t="shared" ref="J207:J211" si="9">B207</f>
+        <f t="shared" ref="J207:J211" si="8">B207</f>
         <v>3.1561896135265709E-5</v>
       </c>
       <c r="K207" s="6">
@@ -4820,7 +4820,7 @@
         <v>5</v>
       </c>
       <c r="J208" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>3.2600000000000001E-6</v>
       </c>
       <c r="K208" s="6">
@@ -4856,7 +4856,7 @@
         <v>5</v>
       </c>
       <c r="J209" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1.2139190821256042E-7</v>
       </c>
       <c r="K209" s="6">
@@ -4892,7 +4892,7 @@
         <v>5</v>
       </c>
       <c r="J210" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>4.9770682367149768E-6</v>
       </c>
       <c r="K210" s="6">
@@ -4928,7 +4928,7 @@
         <v>5</v>
       </c>
       <c r="J211" s="6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>3.6417572463768126E-7</v>
       </c>
       <c r="K211" s="6">
@@ -5321,7 +5321,7 @@
         <v>5</v>
       </c>
       <c r="J237" s="6">
-        <f t="shared" ref="J237:J242" si="10">B237</f>
+        <f t="shared" ref="J237:J242" si="9">B237</f>
         <v>1.0925271739130437E-5</v>
       </c>
       <c r="K237" s="6">
@@ -5357,7 +5357,7 @@
         <v>5</v>
       </c>
       <c r="J238" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>3.1561896135265709E-5</v>
       </c>
       <c r="K238" s="6">
@@ -5393,7 +5393,7 @@
         <v>5</v>
       </c>
       <c r="J239" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>3.2600000000000001E-6</v>
       </c>
       <c r="K239" s="6">
@@ -5429,7 +5429,7 @@
         <v>5</v>
       </c>
       <c r="J240" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>1.2139190821256042E-7</v>
       </c>
       <c r="K240" s="6">
@@ -5465,7 +5465,7 @@
         <v>5</v>
       </c>
       <c r="J241" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>4.9770682367149768E-6</v>
       </c>
       <c r="K241" s="6">
@@ -5501,7 +5501,7 @@
         <v>5</v>
       </c>
       <c r="J242" s="6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>3.6417572463768126E-7</v>
       </c>
       <c r="K242" s="6">
@@ -5894,7 +5894,7 @@
         <v>5</v>
       </c>
       <c r="J268" s="6">
-        <f t="shared" ref="J268:J273" si="11">B268</f>
+        <f t="shared" ref="J268:J273" si="10">B268</f>
         <v>1.0925271739130437E-5</v>
       </c>
       <c r="K268" s="6">
@@ -5930,7 +5930,7 @@
         <v>5</v>
       </c>
       <c r="J269" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>3.1561896135265709E-5</v>
       </c>
       <c r="K269" s="6">
@@ -5966,7 +5966,7 @@
         <v>5</v>
       </c>
       <c r="J270" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>3.2600000000000001E-6</v>
       </c>
       <c r="K270" s="6">
@@ -6002,7 +6002,7 @@
         <v>5</v>
       </c>
       <c r="J271" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1.2139190821256042E-7</v>
       </c>
       <c r="K271" s="6">
@@ -6038,7 +6038,7 @@
         <v>5</v>
       </c>
       <c r="J272" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>4.9770682367149768E-6</v>
       </c>
       <c r="K272" s="6">
@@ -6074,7 +6074,7 @@
         <v>5</v>
       </c>
       <c r="J273" s="6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>3.6417572463768126E-7</v>
       </c>
       <c r="K273" s="6">

</xml_diff>

<commit_message>
Consolidate shared vehicle component inventories
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-ships.xlsx
+++ b/premise/data/additional_inventories/lci-ships.xlsx
@@ -125,10 +125,10 @@
     <t>fuel cell system, 1 kWe, proton exchange membrane (PEM)</t>
   </si>
   <si>
-    <t>fuel tank assembly, compressed hydrogen gas, 700bar</t>
-  </si>
-  <si>
-    <t>fuel tank, compressed hydrogen gas, 700bar</t>
+    <t>fuel tank, compressed hydrogen gas, 700bar, with HDPE liner</t>
+  </si>
+  <si>
+    <t>hydrogen tank</t>
   </si>
   <si>
     <t>market for battery capacity (MIX scenario)</t>
@@ -1043,9 +1043,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O273"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="62.1640625" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
@@ -1056,7 +1056,7 @@
     <col min="10" max="12" width="11.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="16" ns3:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1064,7 +1064,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ns3:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1072,7 +1072,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="16" ns3:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1080,7 +1080,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" ns3:dyDescent="0.2">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" ns3:dyDescent="0.2">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1096,7 +1096,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" ns3:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" ns3:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1112,7 +1112,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" ns3:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" ns3:dyDescent="0.2">
       <c r="A10" t="s">
         <v>91</v>
       </c>
@@ -1129,7 +1129,7 @@
         <v>121500000000.00002</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" ns3:dyDescent="0.2">
       <c r="A11" t="s">
         <v>92</v>
       </c>
@@ -1138,7 +1138,7 @@
         <v>108000000000</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" ns3:dyDescent="0.2">
       <c r="A12" t="s">
         <v>93</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>135000000000</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" ns3:dyDescent="0.2">
       <c r="A13" t="s">
         <v>153</v>
       </c>
@@ -1156,7 +1156,7 @@
         <v>0.32500000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" ns3:dyDescent="0.2">
       <c r="A14" t="s">
         <v>154</v>
       </c>
@@ -1165,7 +1165,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" ns3:dyDescent="0.2">
       <c r="A15" t="s">
         <v>155</v>
       </c>
@@ -1174,7 +1174,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" ns3:dyDescent="0.2">
       <c r="A16" t="s">
         <v>131</v>
       </c>
@@ -1183,7 +1183,7 @@
         <v>0.42500000000000004</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" ns3:dyDescent="0.2">
       <c r="A17" t="s">
         <v>128</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>0.47500000000000003</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" ns3:dyDescent="0.2">
       <c r="A18" t="s">
         <v>129</v>
       </c>
@@ -1201,7 +1201,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" ns3:dyDescent="0.2">
       <c r="A19" t="s">
         <v>130</v>
       </c>
@@ -1210,12 +1210,12 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" ht="16" ns3:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" ns3:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>13</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" ns3:dyDescent="0.2">
       <c r="A22" t="str">
         <f>B4</f>
         <v>transport, freight, sea, container ship, powered with hydrogen</v>
@@ -1276,7 +1276,7 @@
         <v>transport, freight, sea, container ship</v>
       </c>
     </row>
-    <row r="23" spans="1:15" s="5" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" s="5" customFormat="1" ht="16" ns3:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>40</v>
       </c>
@@ -1317,7 +1317,7 @@
       <c r="M23"/>
       <c r="O23" s="7"/>
     </row>
-    <row r="24" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" ht="16" ns3:dyDescent="0.2">
       <c r="A24" s="8" t="s">
         <v>27</v>
       </c>
@@ -1356,7 +1356,7 @@
         <v>2.3148148148148148E-8</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" ns3:dyDescent="0.2">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>2.7777777777777779E-6</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" ns3:dyDescent="0.2">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -1434,7 +1434,7 @@
         <v>9.2592592592592591E-6</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" ns3:dyDescent="0.2">
       <c r="A27" t="s">
         <v>44</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>9.2592592592592589E-12</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" ns3:dyDescent="0.2">
       <c r="A28" t="s">
         <v>50</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>9.2592592592592589E-12</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" ns3:dyDescent="0.2">
       <c r="A29" t="s">
         <v>52</v>
       </c>
@@ -1536,7 +1536,7 @@
       <c r="K29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" ns3:dyDescent="0.2">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -1561,10 +1561,10 @@
       <c r="K30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" ns3:dyDescent="0.2">
       <c r="B31" s="11"/>
     </row>
-    <row r="32" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" ht="16" ns3:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>3</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" ns3:dyDescent="0.2">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" ns3:dyDescent="0.2">
       <c r="A34" t="s">
         <v>10</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" ns3:dyDescent="0.2">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -1596,7 +1596,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" ns3:dyDescent="0.2">
       <c r="A36" t="s">
         <v>6</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" ns3:dyDescent="0.2">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -1612,7 +1612,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" ns3:dyDescent="0.2">
       <c r="A38" t="s">
         <v>91</v>
       </c>
@@ -1621,7 +1621,7 @@
         <v>90000000000</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" ns3:dyDescent="0.2">
       <c r="A39" t="s">
         <v>92</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>72000000000</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" ns3:dyDescent="0.2">
       <c r="A40" t="s">
         <v>93</v>
       </c>
@@ -1639,7 +1639,7 @@
         <v>108000000000</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" ns3:dyDescent="0.2">
       <c r="A41" t="s">
         <v>153</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" ns3:dyDescent="0.2">
       <c r="A42" t="s">
         <v>154</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" ns3:dyDescent="0.2">
       <c r="A43" t="s">
         <v>155</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" ns3:dyDescent="0.2">
       <c r="A44" t="s">
         <v>131</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>0.42500000000000004</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" ns3:dyDescent="0.2">
       <c r="A45" t="s">
         <v>128</v>
       </c>
@@ -1684,7 +1684,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" ns3:dyDescent="0.2">
       <c r="A46" t="s">
         <v>129</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" ns3:dyDescent="0.2">
       <c r="A47" t="s">
         <v>130</v>
       </c>
@@ -1702,12 +1702,12 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" ht="16" ns3:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" ns3:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>13</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" ns3:dyDescent="0.2">
       <c r="A50" t="str">
         <f>B32</f>
         <v>transport, freight, sea, container ship, powered with electricity</v>
@@ -1768,7 +1768,7 @@
         <v>transport, freight, sea, container ship</v>
       </c>
     </row>
-    <row r="51" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A51" t="s">
         <v>151</v>
       </c>
@@ -1807,7 +1807,7 @@
         <v>4.3287037037037041E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" ns3:dyDescent="0.2">
       <c r="A52" t="s">
         <v>31</v>
       </c>
@@ -1846,7 +1846,7 @@
         <v>1.3888888888888889E-4</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12" ns3:dyDescent="0.2">
       <c r="A53" t="s">
         <v>44</v>
       </c>
@@ -1885,7 +1885,7 @@
         <v>1.3888888888888888E-11</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:12" ns3:dyDescent="0.2">
       <c r="A54" t="s">
         <v>50</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>1.3888888888888888E-11</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" ns3:dyDescent="0.2">
       <c r="A55" t="s">
         <v>52</v>
       </c>
@@ -1948,7 +1948,7 @@
       <c r="K55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="57" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>3</v>
       </c>
@@ -1956,7 +1956,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:12" ns3:dyDescent="0.2">
       <c r="A58" t="s">
         <v>11</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:12" ns3:dyDescent="0.2">
       <c r="A59" t="s">
         <v>10</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:12" ns3:dyDescent="0.2">
       <c r="A60" t="s">
         <v>4</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:12" ns3:dyDescent="0.2">
       <c r="A61" t="s">
         <v>6</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:12" ns3:dyDescent="0.2">
       <c r="A62" t="s">
         <v>8</v>
       </c>
@@ -1996,7 +1996,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:12" ns3:dyDescent="0.2">
       <c r="A63" t="s">
         <v>91</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>144000000000</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:12" ns3:dyDescent="0.2">
       <c r="A64" t="s">
         <v>92</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>135000000000</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:12" ns3:dyDescent="0.2">
       <c r="A65" t="s">
         <v>93</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>153000000000</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:12" ns3:dyDescent="0.2">
       <c r="A66" t="s">
         <v>153</v>
       </c>
@@ -2032,7 +2032,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:12" ns3:dyDescent="0.2">
       <c r="A67" t="s">
         <v>154</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:12" ns3:dyDescent="0.2">
       <c r="A68" t="s">
         <v>155</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:12" ns3:dyDescent="0.2">
       <c r="A69" t="s">
         <v>131</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>0.42500000000000004</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:12" ns3:dyDescent="0.2">
       <c r="A70" t="s">
         <v>128</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>0.44020542920029343</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:12" ns3:dyDescent="0.2">
       <c r="A71" t="s">
         <v>129</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:12" ns3:dyDescent="0.2">
       <c r="A72" t="s">
         <v>130</v>
       </c>
@@ -2086,12 +2086,12 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="73" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:12" ns3:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>13</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:12" ns3:dyDescent="0.2">
       <c r="A75" t="str">
         <f>B57</f>
         <v>transport, freight, sea, container ship, powered with liquid ammonia</v>
@@ -2152,7 +2152,7 @@
         <v>transport, freight, sea, container ship</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A76" t="s">
         <v>199</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>9.5750128008192537E-3</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:12" ns3:dyDescent="0.2">
       <c r="A77" t="s">
         <v>31</v>
       </c>
@@ -2230,7 +2230,7 @@
         <v>7.4074074074074073E-8</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:12" ns3:dyDescent="0.2">
       <c r="A78" t="s">
         <v>44</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>7.4074074074074068E-12</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:12" ns3:dyDescent="0.2">
       <c r="A79" t="s">
         <v>50</v>
       </c>
@@ -2308,7 +2308,7 @@
         <v>7.4074074074074068E-12</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:12" ns3:dyDescent="0.2">
       <c r="A80" t="s">
         <v>52</v>
       </c>
@@ -2332,7 +2332,7 @@
       <c r="K80" s="11"/>
       <c r="L80" s="11"/>
     </row>
-    <row r="81" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A81" t="s">
         <v>60</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>2.1571959635416667E-6</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A82" t="s">
         <v>24</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>4.3143919270833341E-5</v>
       </c>
     </row>
-    <row r="83" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A83" t="s">
         <v>61</v>
       </c>
@@ -2440,7 +2440,7 @@
         <v>3.3187630208333344E-7</v>
       </c>
     </row>
-    <row r="84" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A84" t="s">
         <v>62</v>
       </c>
@@ -2476,7 +2476,7 @@
         <v>4.6462682291666672E-8</v>
       </c>
     </row>
-    <row r="85" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A85" t="s">
         <v>25</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>6.6375260416666688E-7</v>
       </c>
     </row>
-    <row r="86" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A86" t="s">
         <v>112</v>
       </c>
@@ -2548,11 +2548,11 @@
         <v>2.1571959635416667E-6</v>
       </c>
     </row>
-    <row r="87" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="J87" s="6"/>
       <c r="K87" s="11"/>
     </row>
-    <row r="88" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>3</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:12" ns3:dyDescent="0.2">
       <c r="A89" t="s">
         <v>11</v>
       </c>
@@ -2568,7 +2568,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:12" ns3:dyDescent="0.2">
       <c r="A90" t="s">
         <v>10</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:12" ns3:dyDescent="0.2">
       <c r="A91" t="s">
         <v>4</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:12" ns3:dyDescent="0.2">
       <c r="A92" t="s">
         <v>6</v>
       </c>
@@ -2592,7 +2592,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:12" ns3:dyDescent="0.2">
       <c r="A93" t="s">
         <v>8</v>
       </c>
@@ -2600,7 +2600,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:12" ns3:dyDescent="0.2">
       <c r="A94" t="s">
         <v>91</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>144000000000</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:12" ns3:dyDescent="0.2">
       <c r="A95" t="s">
         <v>92</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>135000000000</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:12" ns3:dyDescent="0.2">
       <c r="A96" t="s">
         <v>93</v>
       </c>
@@ -2627,7 +2627,7 @@
         <v>153000000000</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:12" ns3:dyDescent="0.2">
       <c r="A97" t="s">
         <v>153</v>
       </c>
@@ -2636,7 +2636,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:12" ns3:dyDescent="0.2">
       <c r="A98" t="s">
         <v>154</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:12" ns3:dyDescent="0.2">
       <c r="A99" t="s">
         <v>155</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:12" ns3:dyDescent="0.2">
       <c r="A100" t="s">
         <v>131</v>
       </c>
@@ -2663,7 +2663,7 @@
         <v>0.42500000000000004</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:12" ns3:dyDescent="0.2">
       <c r="A101" t="s">
         <v>128</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>0.4369674459252787</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:12" ns3:dyDescent="0.2">
       <c r="A102" t="s">
         <v>129</v>
       </c>
@@ -2681,7 +2681,7 @@
         <v>0.32772558444395905</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:12" ns3:dyDescent="0.2">
       <c r="A103" t="s">
         <v>130</v>
       </c>
@@ -2690,12 +2690,12 @@
         <v>0.54620930740659834</v>
       </c>
     </row>
-    <row r="104" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:12" ns3:dyDescent="0.2">
       <c r="A105" s="2" t="s">
         <v>13</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:12" ns3:dyDescent="0.2">
       <c r="A106" t="str">
         <f>B88</f>
         <v>transport, freight, sea, container ship, powered with methanol</v>
@@ -2756,7 +2756,7 @@
         <v>transport, freight, sea, container ship</v>
       </c>
     </row>
-    <row r="107" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A107" t="s">
         <v>198</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>9.5577777777777744E-3</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:12" ns3:dyDescent="0.2">
       <c r="A108" t="s">
         <v>44</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>7.4074074074074068E-12</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:12" ns3:dyDescent="0.2">
       <c r="A109" t="s">
         <v>50</v>
       </c>
@@ -2873,7 +2873,7 @@
         <v>7.4074074074074068E-12</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:12" ns3:dyDescent="0.2">
       <c r="A110" t="s">
         <v>52</v>
       </c>
@@ -2897,7 +2897,7 @@
       <c r="K110" s="11"/>
       <c r="L110" s="11"/>
     </row>
-    <row r="111" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A111" t="s">
         <v>67</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>1.3094155555555553E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A112" t="s">
         <v>60</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>9.7395833333333313E-5</v>
       </c>
     </row>
-    <row r="113" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A113" t="s">
         <v>24</v>
       </c>
@@ -3005,7 +3005,7 @@
         <v>1.8722790624999997E-4</v>
       </c>
     </row>
-    <row r="114" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A114" t="s">
         <v>61</v>
       </c>
@@ -3041,7 +3041,7 @@
         <v>8.4071109374999985E-5</v>
       </c>
     </row>
-    <row r="115" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A115" t="s">
         <v>26</v>
       </c>
@@ -3077,12 +3077,12 @@
         <v>9.9424913194444421E-9</v>
       </c>
     </row>
-    <row r="116" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="J116" s="6"/>
       <c r="K116" s="6"/>
       <c r="L116" s="6"/>
     </row>
-    <row r="117" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>3</v>
       </c>
@@ -3090,7 +3090,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:12" ns3:dyDescent="0.2">
       <c r="A118" t="s">
         <v>11</v>
       </c>
@@ -3098,7 +3098,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:12" ns3:dyDescent="0.2">
       <c r="A119" t="s">
         <v>10</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:12" ns3:dyDescent="0.2">
       <c r="A120" t="s">
         <v>4</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:12" ns3:dyDescent="0.2">
       <c r="A121" t="s">
         <v>6</v>
       </c>
@@ -3122,7 +3122,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:12" ns3:dyDescent="0.2">
       <c r="A122" t="s">
         <v>8</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:12" ns3:dyDescent="0.2">
       <c r="A123" t="s">
         <v>91</v>
       </c>
@@ -3139,7 +3139,7 @@
         <v>108000000000</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:12" ns3:dyDescent="0.2">
       <c r="A124" t="s">
         <v>92</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>90000000000</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:12" ns3:dyDescent="0.2">
       <c r="A125" t="s">
         <v>93</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>117000000000</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:12" ns3:dyDescent="0.2">
       <c r="A126" t="s">
         <v>153</v>
       </c>
@@ -3166,7 +3166,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:12" ns3:dyDescent="0.2">
       <c r="A127" t="s">
         <v>154</v>
       </c>
@@ -3175,7 +3175,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:12" ns3:dyDescent="0.2">
       <c r="A128" t="s">
         <v>155</v>
       </c>
@@ -3184,7 +3184,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:12" ns3:dyDescent="0.2">
       <c r="A129" t="s">
         <v>131</v>
       </c>
@@ -3193,7 +3193,7 @@
         <v>0.42500000000000004</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:12" ns3:dyDescent="0.2">
       <c r="A130" t="s">
         <v>128</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>0.49342105263157898</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:12" ns3:dyDescent="0.2">
       <c r="A131" t="s">
         <v>129</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>0.44407894736842107</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:12" ns3:dyDescent="0.2">
       <c r="A132" t="s">
         <v>130</v>
       </c>
@@ -3220,12 +3220,12 @@
         <v>0.54276315789473695</v>
       </c>
     </row>
-    <row r="133" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:12" ns3:dyDescent="0.2">
       <c r="A134" s="2" t="s">
         <v>13</v>
       </c>
@@ -3263,7 +3263,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:12" ns3:dyDescent="0.2">
       <c r="A135" t="str">
         <f>B117</f>
         <v>transport, freight, sea, container ship, powered with synthetic methane</v>
@@ -3286,7 +3286,7 @@
         <v>transport, freight, sea, container ship</v>
       </c>
     </row>
-    <row r="136" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A136" t="s">
         <v>107</v>
       </c>
@@ -3325,7 +3325,7 @@
         <v>4.432592592592593E-3</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:12" ns3:dyDescent="0.2">
       <c r="A137" t="s">
         <v>44</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>1.1111111111111111E-11</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:12" ns3:dyDescent="0.2">
       <c r="A138" t="s">
         <v>50</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>1.1111111111111111E-11</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:12" ns3:dyDescent="0.2">
       <c r="A139" t="s">
         <v>52</v>
       </c>
@@ -3427,7 +3427,7 @@
       <c r="K139" s="11"/>
       <c r="L139" s="11"/>
     </row>
-    <row r="140" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A140" t="s">
         <v>67</v>
       </c>
@@ -3463,7 +3463,7 @@
         <v>1.2145303703703706E-2</v>
       </c>
     </row>
-    <row r="141" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A141" t="s">
         <v>60</v>
       </c>
@@ -3499,7 +3499,7 @@
         <v>4.4748771929824572E-5</v>
       </c>
     </row>
-    <row r="142" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A142" t="s">
         <v>24</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>2.8148421052631585E-5</v>
       </c>
     </row>
-    <row r="143" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A143" t="s">
         <v>110</v>
       </c>
@@ -3571,7 +3571,7 @@
         <v>7.2175438596491244E-7</v>
       </c>
     </row>
-    <row r="144" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A144" t="s">
         <v>61</v>
       </c>
@@ -3607,7 +3607,7 @@
         <v>7.2175438596491244E-7</v>
       </c>
     </row>
-    <row r="145" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A145" t="s">
         <v>111</v>
       </c>
@@ -3643,7 +3643,7 @@
         <v>2.2273777777777779E-4</v>
       </c>
     </row>
-    <row r="146" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A146" t="s">
         <v>62</v>
       </c>
@@ -3679,7 +3679,7 @@
         <v>9.1422222222222249E-6</v>
       </c>
     </row>
-    <row r="147" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A147" t="s">
         <v>112</v>
       </c>
@@ -3715,7 +3715,7 @@
         <v>4.81169590643275E-7</v>
       </c>
     </row>
-    <row r="150" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>3</v>
       </c>
@@ -3723,7 +3723,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:12" ns3:dyDescent="0.2">
       <c r="A151" t="s">
         <v>11</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:12" ns3:dyDescent="0.2">
       <c r="A152" t="s">
         <v>10</v>
       </c>
@@ -3739,7 +3739,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:12" ns3:dyDescent="0.2">
       <c r="A153" t="s">
         <v>4</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:12" ns3:dyDescent="0.2">
       <c r="A154" t="s">
         <v>6</v>
       </c>
@@ -3755,7 +3755,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:12" ns3:dyDescent="0.2">
       <c r="A155" t="s">
         <v>8</v>
       </c>
@@ -3763,7 +3763,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:12" ns3:dyDescent="0.2">
       <c r="A156" t="s">
         <v>91</v>
       </c>
@@ -3772,7 +3772,7 @@
         <v>163923092656.98508</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:12" ns3:dyDescent="0.2">
       <c r="A157" t="s">
         <v>92</v>
       </c>
@@ -3781,7 +3781,7 @@
         <v>159903865821.23132</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:12" ns3:dyDescent="0.2">
       <c r="A158" t="s">
         <v>93</v>
       </c>
@@ -3790,7 +3790,7 @@
         <v>166602577214.15421</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:12" ns3:dyDescent="0.2">
       <c r="A159" t="s">
         <v>153</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>8.9316151905638519E-2</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:12" ns3:dyDescent="0.2">
       <c r="A160" t="s">
         <v>154</v>
       </c>
@@ -3808,7 +3808,7 @@
         <v>7.4430126588032122E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:12" ns3:dyDescent="0.2">
       <c r="A161" t="s">
         <v>155</v>
       </c>
@@ -3817,7 +3817,7 @@
         <v>0.11164518988204816</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:12" ns3:dyDescent="0.2">
       <c r="A162" t="s">
         <v>131</v>
       </c>
@@ -3826,7 +3826,7 @@
         <v>0.42500000000000004</v>
       </c>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:12" ns3:dyDescent="0.2">
       <c r="A163" t="s">
         <v>128</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>0.49342105263157898</v>
       </c>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:12" ns3:dyDescent="0.2">
       <c r="A164" t="s">
         <v>129</v>
       </c>
@@ -3844,7 +3844,7 @@
         <v>0.44407894736842107</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:12" ns3:dyDescent="0.2">
       <c r="A165" t="s">
         <v>130</v>
       </c>
@@ -3853,12 +3853,12 @@
         <v>0.54276315789473695</v>
       </c>
     </row>
-    <row r="166" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A166" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:12" ns3:dyDescent="0.2">
       <c r="A167" s="2" t="s">
         <v>13</v>
       </c>
@@ -3896,7 +3896,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:12" ns3:dyDescent="0.2">
       <c r="A168" t="str">
         <f>B150</f>
         <v>transport, freight, sea, container ship, powered with synthetic liquefied petroleum gas</v>
@@ -3919,7 +3919,7 @@
         <v>transport, freight, sea, container ship</v>
       </c>
     </row>
-    <row r="169" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A169" t="s">
         <v>197</v>
       </c>
@@ -3958,7 +3958,7 @@
         <v>2.5761855529249592E-3</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:12" ns3:dyDescent="0.2">
       <c r="A170" t="s">
         <v>44</v>
       </c>
@@ -3997,7 +3997,7 @@
         <v>6.25375749900866E-12</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:12" ns3:dyDescent="0.2">
       <c r="A171" t="s">
         <v>50</v>
       </c>
@@ -4036,7 +4036,7 @@
         <v>6.25375749900866E-12</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:12" ns3:dyDescent="0.2">
       <c r="A172" t="s">
         <v>52</v>
       </c>
@@ -4060,7 +4060,7 @@
       <c r="K172" s="11"/>
       <c r="L172" s="11"/>
     </row>
-    <row r="173" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A173" t="s">
         <v>67</v>
       </c>
@@ -4096,7 +4096,7 @@
         <v>7.7285566587748777E-3</v>
       </c>
     </row>
-    <row r="174" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A174" t="s">
         <v>60</v>
       </c>
@@ -4132,7 +4132,7 @@
         <v>2.9175419536572591E-5</v>
       </c>
     </row>
-    <row r="175" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A175" t="s">
         <v>24</v>
       </c>
@@ -4168,7 +4168,7 @@
         <v>1.8352280031069855E-5</v>
       </c>
     </row>
-    <row r="176" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A176" t="s">
         <v>110</v>
       </c>
@@ -4204,7 +4204,7 @@
         <v>4.7057128284794499E-7</v>
       </c>
     </row>
-    <row r="177" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A177" t="s">
         <v>61</v>
       </c>
@@ -4240,7 +4240,7 @@
         <v>4.7057128284794499E-7</v>
       </c>
     </row>
-    <row r="178" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A178" t="s">
         <v>111</v>
       </c>
@@ -4276,7 +4276,7 @@
         <v>1.5153511287030737E-4</v>
       </c>
     </row>
-    <row r="179" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A179" t="s">
         <v>62</v>
       </c>
@@ -4312,7 +4312,7 @@
         <v>5.9605695827406364E-6</v>
       </c>
     </row>
-    <row r="180" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A180" t="s">
         <v>112</v>
       </c>
@@ -4348,7 +4348,7 @@
         <v>3.1371418856529668E-7</v>
       </c>
     </row>
-    <row r="182" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A182" s="1" t="s">
         <v>3</v>
       </c>
@@ -4356,7 +4356,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:12" ns3:dyDescent="0.2">
       <c r="A183" t="s">
         <v>11</v>
       </c>
@@ -4364,7 +4364,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:12" ns3:dyDescent="0.2">
       <c r="A184" t="s">
         <v>10</v>
       </c>
@@ -4372,7 +4372,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:12" ns3:dyDescent="0.2">
       <c r="A185" t="s">
         <v>4</v>
       </c>
@@ -4380,7 +4380,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:12" ns3:dyDescent="0.2">
       <c r="A186" t="s">
         <v>6</v>
       </c>
@@ -4388,7 +4388,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:12" ns3:dyDescent="0.2">
       <c r="A187" t="s">
         <v>8</v>
       </c>
@@ -4396,7 +4396,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:12" ns3:dyDescent="0.2">
       <c r="A188" t="s">
         <v>91</v>
       </c>
@@ -4405,7 +4405,7 @@
         <v>180000000000</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:12" ns3:dyDescent="0.2">
       <c r="A189" t="s">
         <v>92</v>
       </c>
@@ -4414,7 +4414,7 @@
         <v>180000000000</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:12" ns3:dyDescent="0.2">
       <c r="A190" t="s">
         <v>93</v>
       </c>
@@ -4423,7 +4423,7 @@
         <v>180000000000</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:12" ns3:dyDescent="0.2">
       <c r="A191" t="s">
         <v>153</v>
       </c>
@@ -4431,7 +4431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:12" ns3:dyDescent="0.2">
       <c r="A192" t="s">
         <v>154</v>
       </c>
@@ -4439,7 +4439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:12" ns3:dyDescent="0.2">
       <c r="A193" t="s">
         <v>155</v>
       </c>
@@ -4447,7 +4447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:12" ns3:dyDescent="0.2">
       <c r="A194" t="s">
         <v>131</v>
       </c>
@@ -4456,7 +4456,7 @@
         <v>0.42500000000000004</v>
       </c>
     </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:12" ns3:dyDescent="0.2">
       <c r="A195" t="s">
         <v>128</v>
       </c>
@@ -4465,7 +4465,7 @@
         <v>0.50434295320818157</v>
       </c>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:12" ns3:dyDescent="0.2">
       <c r="A196" t="s">
         <v>129</v>
       </c>
@@ -4474,7 +4474,7 @@
         <v>0.4539086578873634</v>
       </c>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:12" ns3:dyDescent="0.2">
       <c r="A197" t="s">
         <v>130</v>
       </c>
@@ -4483,12 +4483,12 @@
         <v>0.55477724852899979</v>
       </c>
     </row>
-    <row r="198" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A198" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:12" ns3:dyDescent="0.2">
       <c r="A199" s="2" t="s">
         <v>13</v>
       </c>
@@ -4526,7 +4526,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:12" ns3:dyDescent="0.2">
       <c r="A200" t="str">
         <f>B182</f>
         <v>transport, freight, sea, container ship, powered with diesel</v>
@@ -4549,7 +4549,7 @@
         <v>transport, freight, sea, container ship</v>
       </c>
     </row>
-    <row r="201" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A201" t="s">
         <v>173</v>
       </c>
@@ -4588,7 +4588,7 @@
         <v>2.2390063070316696E-3</v>
       </c>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:12" ns3:dyDescent="0.2">
       <c r="A202" t="s">
         <v>44</v>
       </c>
@@ -4615,7 +4615,7 @@
       <c r="K202" s="11"/>
       <c r="L202" s="11"/>
     </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:12" ns3:dyDescent="0.2">
       <c r="A203" t="s">
         <v>50</v>
       </c>
@@ -4642,7 +4642,7 @@
       <c r="K203" s="11"/>
       <c r="L203" s="11"/>
     </row>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:12" ns3:dyDescent="0.2">
       <c r="A204" t="s">
         <v>52</v>
       </c>
@@ -4666,7 +4666,7 @@
       <c r="K204" s="11"/>
       <c r="L204" s="11"/>
     </row>
-    <row r="205" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A205" t="s">
         <v>170</v>
       </c>
@@ -4702,7 +4702,7 @@
         <v>6.7170189210950092E-3</v>
       </c>
     </row>
-    <row r="206" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A206" t="s">
         <v>171</v>
       </c>
@@ -4738,7 +4738,7 @@
         <v>1.2017798913043482E-5</v>
       </c>
     </row>
-    <row r="207" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A207" t="s">
         <v>24</v>
       </c>
@@ -4774,7 +4774,7 @@
         <v>3.4718085748792285E-5</v>
       </c>
     </row>
-    <row r="208" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A208" t="s">
         <v>61</v>
       </c>
@@ -4810,7 +4810,7 @@
         <v>6.5200000000000003E-6</v>
       </c>
     </row>
-    <row r="209" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A209" t="s">
         <v>172</v>
       </c>
@@ -4846,7 +4846,7 @@
         <v>1.3353109903381649E-7</v>
       </c>
     </row>
-    <row r="210" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A210" t="s">
         <v>62</v>
       </c>
@@ -4882,7 +4882,7 @@
         <v>5.3412439613526591E-6</v>
       </c>
     </row>
-    <row r="211" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A211" t="s">
         <v>112</v>
       </c>
@@ -4918,7 +4918,7 @@
         <v>4.0059329710144941E-7</v>
       </c>
     </row>
-    <row r="213" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A213" s="1" t="s">
         <v>3</v>
       </c>
@@ -4926,7 +4926,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:12" ns3:dyDescent="0.2">
       <c r="A214" t="s">
         <v>11</v>
       </c>
@@ -4934,7 +4934,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:12" ns3:dyDescent="0.2">
       <c r="A215" t="s">
         <v>10</v>
       </c>
@@ -4942,7 +4942,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:12" ns3:dyDescent="0.2">
       <c r="A216" t="s">
         <v>4</v>
       </c>
@@ -4950,7 +4950,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:12" ns3:dyDescent="0.2">
       <c r="A217" t="s">
         <v>6</v>
       </c>
@@ -4958,7 +4958,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:12" ns3:dyDescent="0.2">
       <c r="A218" t="s">
         <v>8</v>
       </c>
@@ -4966,7 +4966,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:12" ns3:dyDescent="0.2">
       <c r="A219" t="s">
         <v>91</v>
       </c>
@@ -4975,7 +4975,7 @@
         <v>180000000000</v>
       </c>
     </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:12" ns3:dyDescent="0.2">
       <c r="A220" t="s">
         <v>92</v>
       </c>
@@ -4984,7 +4984,7 @@
         <v>180000000000</v>
       </c>
     </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:12" ns3:dyDescent="0.2">
       <c r="A221" t="s">
         <v>93</v>
       </c>
@@ -4993,7 +4993,7 @@
         <v>180000000000</v>
       </c>
     </row>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:12" ns3:dyDescent="0.2">
       <c r="A222" t="s">
         <v>153</v>
       </c>
@@ -5002,7 +5002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:12" ns3:dyDescent="0.2">
       <c r="A223" t="s">
         <v>154</v>
       </c>
@@ -5011,7 +5011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:12" ns3:dyDescent="0.2">
       <c r="A224" t="s">
         <v>155</v>
       </c>
@@ -5020,7 +5020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:12" ns3:dyDescent="0.2">
       <c r="A225" t="s">
         <v>131</v>
       </c>
@@ -5029,7 +5029,7 @@
         <v>0.42500000000000004</v>
       </c>
     </row>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:12" ns3:dyDescent="0.2">
       <c r="A226" t="s">
         <v>128</v>
       </c>
@@ -5038,7 +5038,7 @@
         <v>0.50434295320818157</v>
       </c>
     </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:12" ns3:dyDescent="0.2">
       <c r="A227" t="s">
         <v>129</v>
       </c>
@@ -5047,7 +5047,7 @@
         <v>0.4539086578873634</v>
       </c>
     </row>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:12" ns3:dyDescent="0.2">
       <c r="A228" t="s">
         <v>130</v>
       </c>
@@ -5056,12 +5056,12 @@
         <v>0.55477724852899979</v>
       </c>
     </row>
-    <row r="229" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A229" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:12" ns3:dyDescent="0.2">
       <c r="A230" s="2" t="s">
         <v>13</v>
       </c>
@@ -5099,7 +5099,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:12" ns3:dyDescent="0.2">
       <c r="A231" t="str">
         <f>B213</f>
         <v>transport, freight, sea, container ship, powered with synthetic diesel</v>
@@ -5122,7 +5122,7 @@
         <v>transport, freight, sea, container ship</v>
       </c>
     </row>
-    <row r="232" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A232" t="s">
         <v>196</v>
       </c>
@@ -5161,7 +5161,7 @@
         <v>2.2390063070316696E-3</v>
       </c>
     </row>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:12" ns3:dyDescent="0.2">
       <c r="A233" t="s">
         <v>44</v>
       </c>
@@ -5188,7 +5188,7 @@
       <c r="K233" s="11"/>
       <c r="L233" s="11"/>
     </row>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:12" ns3:dyDescent="0.2">
       <c r="A234" t="s">
         <v>50</v>
       </c>
@@ -5215,7 +5215,7 @@
       <c r="K234" s="11"/>
       <c r="L234" s="11"/>
     </row>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:12" ns3:dyDescent="0.2">
       <c r="A235" t="s">
         <v>52</v>
       </c>
@@ -5239,7 +5239,7 @@
       <c r="K235" s="11"/>
       <c r="L235" s="11"/>
     </row>
-    <row r="236" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A236" t="s">
         <v>67</v>
       </c>
@@ -5275,7 +5275,7 @@
         <v>6.7170189210950092E-3</v>
       </c>
     </row>
-    <row r="237" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A237" t="s">
         <v>60</v>
       </c>
@@ -5311,7 +5311,7 @@
         <v>1.2017798913043482E-5</v>
       </c>
     </row>
-    <row r="238" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A238" t="s">
         <v>24</v>
       </c>
@@ -5347,7 +5347,7 @@
         <v>3.4718085748792285E-5</v>
       </c>
     </row>
-    <row r="239" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A239" t="s">
         <v>61</v>
       </c>
@@ -5383,7 +5383,7 @@
         <v>6.5200000000000003E-6</v>
       </c>
     </row>
-    <row r="240" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A240" t="s">
         <v>111</v>
       </c>
@@ -5419,7 +5419,7 @@
         <v>1.3353109903381649E-7</v>
       </c>
     </row>
-    <row r="241" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A241" t="s">
         <v>62</v>
       </c>
@@ -5455,7 +5455,7 @@
         <v>5.4747750603864751E-6</v>
       </c>
     </row>
-    <row r="242" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A242" t="s">
         <v>112</v>
       </c>
@@ -5491,7 +5491,7 @@
         <v>4.0059329710144941E-7</v>
       </c>
     </row>
-    <row r="244" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A244" s="1" t="s">
         <v>3</v>
       </c>
@@ -5499,7 +5499,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:12" ns3:dyDescent="0.2">
       <c r="A245" t="s">
         <v>11</v>
       </c>
@@ -5507,7 +5507,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:12" ns3:dyDescent="0.2">
       <c r="A246" t="s">
         <v>10</v>
       </c>
@@ -5515,7 +5515,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:12" ns3:dyDescent="0.2">
       <c r="A247" t="s">
         <v>4</v>
       </c>
@@ -5523,7 +5523,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:12" ns3:dyDescent="0.2">
       <c r="A248" t="s">
         <v>6</v>
       </c>
@@ -5531,7 +5531,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:12" ns3:dyDescent="0.2">
       <c r="A249" t="s">
         <v>8</v>
       </c>
@@ -5539,7 +5539,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:12" ns3:dyDescent="0.2">
       <c r="A250" t="s">
         <v>91</v>
       </c>
@@ -5548,7 +5548,7 @@
         <v>180000000000</v>
       </c>
     </row>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:12" ns3:dyDescent="0.2">
       <c r="A251" t="s">
         <v>92</v>
       </c>
@@ -5557,7 +5557,7 @@
         <v>180000000000</v>
       </c>
     </row>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:12" ns3:dyDescent="0.2">
       <c r="A252" t="s">
         <v>93</v>
       </c>
@@ -5566,7 +5566,7 @@
         <v>180000000000</v>
       </c>
     </row>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:12" ns3:dyDescent="0.2">
       <c r="A253" t="s">
         <v>153</v>
       </c>
@@ -5575,7 +5575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:12" ns3:dyDescent="0.2">
       <c r="A254" t="s">
         <v>154</v>
       </c>
@@ -5584,7 +5584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:12" ns3:dyDescent="0.2">
       <c r="A255" t="s">
         <v>155</v>
       </c>
@@ -5593,7 +5593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:12" ns3:dyDescent="0.2">
       <c r="A256" t="s">
         <v>131</v>
       </c>
@@ -5602,7 +5602,7 @@
         <v>0.42500000000000004</v>
       </c>
     </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:12" ns3:dyDescent="0.2">
       <c r="A257" t="s">
         <v>128</v>
       </c>
@@ -5611,7 +5611,7 @@
         <v>0.50434295320818157</v>
       </c>
     </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:12" ns3:dyDescent="0.2">
       <c r="A258" t="s">
         <v>129</v>
       </c>
@@ -5620,7 +5620,7 @@
         <v>0.4539086578873634</v>
       </c>
     </row>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:12" ns3:dyDescent="0.2">
       <c r="A259" t="s">
         <v>130</v>
       </c>
@@ -5629,12 +5629,12 @@
         <v>0.55477724852899979</v>
       </c>
     </row>
-    <row r="260" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A260" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:12" ns3:dyDescent="0.2">
       <c r="A261" s="2" t="s">
         <v>13</v>
       </c>
@@ -5672,7 +5672,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="262" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:12" ns3:dyDescent="0.2">
       <c r="A262" t="str">
         <f>B244</f>
         <v>transport, freight, sea, container ship, powered with biodiesel</v>
@@ -5695,7 +5695,7 @@
         <v>transport, freight, sea, container ship</v>
       </c>
     </row>
-    <row r="263" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A263" t="s">
         <v>168</v>
       </c>
@@ -5734,7 +5734,7 @@
         <v>2.2390063070316696E-3</v>
       </c>
     </row>
-    <row r="264" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:12" ns3:dyDescent="0.2">
       <c r="A264" t="s">
         <v>44</v>
       </c>
@@ -5761,7 +5761,7 @@
       <c r="K264" s="11"/>
       <c r="L264" s="11"/>
     </row>
-    <row r="265" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:12" ns3:dyDescent="0.2">
       <c r="A265" t="s">
         <v>50</v>
       </c>
@@ -5788,7 +5788,7 @@
       <c r="K265" s="11"/>
       <c r="L265" s="11"/>
     </row>
-    <row r="266" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:12" ns3:dyDescent="0.2">
       <c r="A266" t="s">
         <v>52</v>
       </c>
@@ -5812,7 +5812,7 @@
       <c r="K266" s="11"/>
       <c r="L266" s="11"/>
     </row>
-    <row r="267" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A267" t="s">
         <v>67</v>
       </c>
@@ -5848,7 +5848,7 @@
         <v>6.7170189210950092E-3</v>
       </c>
     </row>
-    <row r="268" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A268" t="s">
         <v>60</v>
       </c>
@@ -5884,7 +5884,7 @@
         <v>1.2017798913043482E-5</v>
       </c>
     </row>
-    <row r="269" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A269" t="s">
         <v>24</v>
       </c>
@@ -5920,7 +5920,7 @@
         <v>3.4718085748792285E-5</v>
       </c>
     </row>
-    <row r="270" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A270" t="s">
         <v>61</v>
       </c>
@@ -5956,7 +5956,7 @@
         <v>6.5200000000000003E-6</v>
       </c>
     </row>
-    <row r="271" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A271" t="s">
         <v>111</v>
       </c>
@@ -5992,7 +5992,7 @@
         <v>1.3353109903381649E-7</v>
       </c>
     </row>
-    <row r="272" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A272" t="s">
         <v>62</v>
       </c>
@@ -6028,7 +6028,7 @@
         <v>5.4747750603864751E-6</v>
       </c>
     </row>
-    <row r="273" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:12" ht="16" ns3:dyDescent="0.2">
       <c r="A273" t="s">
         <v>112</v>
       </c>
@@ -6065,7 +6065,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O225" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:O225" ns2:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>